<commit_message>
J02: mise à jour du mini-projet bulletin scolaire
</commit_message>
<xml_diff>
--- a/01-Fondamentaux/J02-Mise-en-forme-essentielle/exercices/Classeur-J02.xlsx
+++ b/01-Fondamentaux/J02-Mise-en-forme-essentielle/exercices/Classeur-J02.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\excel-data-bootcamp\01-Fondamentaux\J02-Mise-en-forme-essentielle\exercices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39658827-B077-40E8-80AA-66279600F7C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{347E9559-4DCF-44A4-8320-D527979F071F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="56">
   <si>
     <t>ID</t>
   </si>
@@ -185,6 +185,15 @@
   </si>
   <si>
     <t>BULLETIN SCOLAIRE 2026 - 2027</t>
+  </si>
+  <si>
+    <t>Matière</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Maths</t>
   </si>
 </sst>
 </file>
@@ -192,13 +201,20 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="#,##0&quot; FCFA&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0&quot; FCFA&quot;"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -268,6 +284,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -301,7 +323,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -361,119 +383,113 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,13 +724,13 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="21"/>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="24"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23"/>
       <c r="H1" s="19"/>
       <c r="I1" s="14"/>
       <c r="J1" s="17"/>
@@ -2248,7 +2264,7 @@
   <mergeCells count="1">
     <mergeCell ref="C1:E1"/>
   </mergeCells>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -2256,102 +2272,131 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D29072-C546-419C-A8D6-3DA0FD7E1C66}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="18.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.81640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="20.6328125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="10.90625" customWidth="1"/>
+    <col min="4" max="4" width="10.90625" style="36"/>
+    <col min="6" max="6" width="15.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.6328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="37" t="s">
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="35" t="s">
+      <c r="B2" s="40"/>
+      <c r="C2" s="41" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="39" t="s">
+      <c r="D2" s="42"/>
+      <c r="E2" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="27" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="27" t="s">
+      <c r="C3" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="27">
+        <v>15.5</v>
+      </c>
+      <c r="E4" s="28">
+        <v>0.95</v>
+      </c>
+      <c r="F4" s="30">
+        <v>75000</v>
+      </c>
+      <c r="G4" s="32">
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="D5" s="45">
+        <v>16.75</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="17"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="33" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="29">
-        <v>15.5</v>
-      </c>
-      <c r="D4" s="29">
-        <v>16.75</v>
-      </c>
-      <c r="E4" s="29">
+      <c r="D6" s="45">
         <v>14</v>
       </c>
-      <c r="F4" s="30">
-        <v>0.95</v>
-      </c>
-      <c r="G4" s="32">
-        <v>75000</v>
-      </c>
-      <c r="H4" s="34">
-        <v>46037</v>
-      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="17"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C2:D2"/>
   </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>